<commit_message>
Ponto de equilibrio com regua de LB, botao Preco planilha | Preco sistema e setembro fechado
- Ponto de equilibrio no topo do Resumo (B2 Centro em foco): numero grande, regua do LB
  (azul cobre os custos, laranja o que passa, listrado o que falta), comparacao com a
  media do posto e da rede, litros/dia para empatar.
- Botao Preco planilha | Preco sistema: desconto do boleto por distribuidora
  (data/descontos_boleto.csv, editor na Administracao); muda margem, LB, perda e equilibrio.
- Painel antigo removido (visual unico); vocabulario LB (Lucro Bruto), menos legendas;
  menu com B2 Centro "(Em Construcao)" no topo e os demais "(construir)".
- Dados simulados: setembro fechado (30/09; so a Primavera para em 27/09); a historia do
  diesel do Candoi (~1 dia de autonomia) recolocada com a entrega atrasada a partir de 22/09.
- Testes novos: equilibrio (18) e descontos (13); 214 passando.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/b2_bonsucesso/B2 Bonsucesso 01-2026.xlsx
+++ b/data/b2_bonsucesso/B2 Bonsucesso 01-2026.xlsx
@@ -4824,164 +4824,164 @@
     </row>
     <row r="2">
       <c r="A2" s="7" t="n">
-        <v>46026</v>
+        <v>46025</v>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Taxas de cartão</t>
+          <t>Manutenção</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Taxas das maquininhas (semana)</t>
+          <t>Reparo elétrico</t>
         </is>
       </c>
       <c r="D2" s="16" t="n">
-        <v>2453.37</v>
+        <v>1275.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="n">
-        <v>46027</v>
+        <v>46026</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Folha de pagamento</t>
+          <t>Taxas de cartão</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Salários do mês anterior</t>
+          <t>Taxas das maquininhas (semana)</t>
         </is>
       </c>
       <c r="D3" s="17" t="n">
-        <v>65543.35000000001</v>
+        <v>2277.07</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
-        <v>46029</v>
+        <v>46027</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Outras despesas</t>
+          <t>Folha de pagamento</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Coleta de resíduos (óleo e borra)</t>
+          <t>Salários do mês anterior</t>
         </is>
       </c>
       <c r="D4" s="16" t="n">
-        <v>1554.76</v>
+        <v>65221.41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="n">
-        <v>46032</v>
+        <v>46028</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sistemas e contabilidade</t>
+          <t>Outras despesas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sistema de automação e contabilidade</t>
+          <t>Seguro do posto</t>
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>3600</v>
+        <v>1318.64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>46033</v>
+        <v>46030</v>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Taxas de cartão</t>
+          <t>Manutenção</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Taxas das maquininhas (semana)</t>
+          <t>Manutenção do compressor de ar</t>
         </is>
       </c>
       <c r="D6" s="16" t="n">
-        <v>3811.71</v>
+        <v>3340.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="n">
-        <v>46034</v>
+        <v>46032</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Água e esgoto</t>
+          <t>Sistemas e contabilidade</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Conta de água</t>
+          <t>Sistema de automação e contabilidade</t>
         </is>
       </c>
       <c r="D7" s="17" t="n">
-        <v>1523.54</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
-        <v>46035</v>
+        <v>46033</v>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Manutenção</t>
+          <t>Taxas de cartão</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Limpeza da caixa separadora</t>
+          <t>Taxas das maquininhas (semana)</t>
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>3549.38</v>
+        <v>4092.35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="n">
-        <v>46035</v>
+        <v>46034</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Manutenção</t>
+          <t>Água e esgoto</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Troca de filtros das bombas</t>
+          <t>Conta de água</t>
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>3620.56</v>
+        <v>1395.54</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>46037</v>
+        <v>46036</v>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Energia elétrica</t>
+          <t>Outras despesas</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Conta de energia</t>
+          <t>Monitoramento e alarme</t>
         </is>
       </c>
       <c r="D10" s="16" t="n">
-        <v>10193.36</v>
+        <v>2219.46</v>
       </c>
     </row>
     <row r="11">
@@ -4990,106 +4990,106 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Energia elétrica</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Placas, redes sociais e brindes</t>
+          <t>Conta de energia</t>
         </is>
       </c>
       <c r="D11" s="17" t="n">
-        <v>2124.89</v>
+        <v>10699.31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
-        <v>46040</v>
+        <v>46037</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Taxas de cartão</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Taxas das maquininhas (semana)</t>
+          <t>Placas, redes sociais e brindes</t>
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>4340.62</v>
+        <v>1929.65</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="n">
-        <v>46042</v>
+        <v>46040</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Folha de pagamento</t>
+          <t>Taxas de cartão</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Encargos (INSS e FGTS)</t>
+          <t>Taxas das maquininhas (semana)</t>
         </is>
       </c>
       <c r="D13" s="17" t="n">
-        <v>22807.67</v>
+        <v>4350.96</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
-        <v>46046</v>
+        <v>46042</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Outras despesas</t>
+          <t>Folha de pagamento</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Material de limpeza e escritório</t>
+          <t>Encargos (INSS e FGTS)</t>
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>1326.32</v>
+        <v>22988.65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="n">
-        <v>46047</v>
+        <v>46044</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Taxas de cartão</t>
+          <t>Outras despesas</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Taxas das maquininhas (semana)</t>
+          <t>Material de limpeza e escritório</t>
         </is>
       </c>
       <c r="D15" s="17" t="n">
-        <v>4008.02</v>
+        <v>1483.43</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>46048</v>
+        <v>46047</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Outras despesas</t>
+          <t>Taxas de cartão</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Seguro do posto</t>
+          <t>Taxas das maquininhas (semana)</t>
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>1778.25</v>
+        <v>4076.53</v>
       </c>
     </row>
     <row r="17">
@@ -5107,7 +5107,7 @@
         </is>
       </c>
       <c r="D17" s="17" t="n">
-        <v>3713.17</v>
+        <v>3721.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>